<commit_message>
Auto commit (2026-09-23 12:09) — 12 changes
Claude Code 세션 종료 시 자동 커밋.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/ee741391-22c8-4881-8ea8-ea99262859e6
</commit_message>
<xml_diff>
--- a/projects/16_moses/내 남편은 거지 모세_CD1 셀링 포인트_v2.xlsx
+++ b/projects/16_moses/내 남편은 거지 모세_CD1 셀링 포인트_v2.xlsx
@@ -23109,7 +23109,7 @@
       </c>
       <c r="H18" s="243" t="inlineStr">
         <is>
-          <t>델릴라가 불길 위에서 펜던트를 흔들며 다말에게 맨발로 불의 길을 걸으라 조롱하고, 다말은 델릴라가 진짜로 펜던트를 불에 던지려 하자 걷겠다고 답한다. 신발을 벗은 다말이 불타는 장작길 위로 발을 내딛고, 살이 타는 고통 속에서도 끝까지 걸어 펜던트를 향해 나아간다. 같은 시각 성소에서 기도하던 모세는 아론에게 다말이 위험하다는 말을 듣고 지팡이로 옷을 신성한 예복으로 바꾼 뒤 모래폭풍을 일으켜 하늘로 솟아오른다.</t>
+          <t>델릴라가 불길 위에서 펜던트를 흔들며 다말에게 맨발로 불의 길을 걸으라 조롱하고, 다말은 델릴라가 펜던트를 불에 던지는 시늉을 하자 걷겠다고 답한다. 신발을 벗은 다말이 불타는 장작길 위로 발을 내딛고, 살이 타는 고통 속에서도 끝까지 걸어 펜던트를 향해 나아간다. 같은 시각 성소에서 기도하던 모세는 아론에게 다말이 위험하다는 말을 듣고 지팡이로 옷을 신성한 예복으로 바꾼 뒤 모래폭풍을 일으켜 하늘로 솟아오른다.</t>
         </is>
       </c>
     </row>
@@ -23121,12 +23121,12 @@
       </c>
       <c r="B19" s="243" t="inlineStr">
         <is>
-          <t>NetShort &lt;Swapped to a Beggar But He is Apollo&gt;(48화)를 모세와 출애굽 세계로 옮긴 각색. 노출과 정사는 9화 첫날밤 한 번(남주 상의 탈의, 드레스 흘러내림, 키스까지). 그 밖의 키스는 23·40·50화.</t>
+          <t>NetShort &lt;Swapped to a Beggar But He is Apollo&gt;(48화)를 모세와 출애굽 세계로 옮긴 각색. 노출과 정사는 9화 첫날밤 한 번(남주 상의 탈의, 드레스 흘러내림, 키스까지). 그 밖의 키스는 10화(이마)·23·40·50화.</t>
         </is>
       </c>
       <c r="C19" s="243" t="inlineStr">
         <is>
-          <t>An adaptation of NetShort's &lt;Swapped to a Beggar But He is Apollo&gt; (48 EP) moved into a Moses / Exodus world. One bedroom scene, the EP9 wedding night (ML shirtless, dress slipping off, kiss). Other kisses in EP23, EP40 and EP50.</t>
+          <t>An adaptation of NetShort's &lt;Swapped to a Beggar But He is Apollo&gt; (48 EP) moved into a Moses / Exodus world. One bedroom scene, the EP9 wedding night (ML shirtless, dress slipping off, kiss). Other kisses in EP10 (forehead), EP23, EP40 and EP50.</t>
         </is>
       </c>
       <c r="F19" s="245" t="n">
@@ -23160,7 +23160,7 @@
       </c>
       <c r="H20" s="243" t="inlineStr">
         <is>
-          <t>모세가 델릴라를 걷어차 쓰러뜨리고 피투성이가 된 다말을 품에 안아 일으킨 뒤 손에 입을 맞춘다. 라반과 네페라는 노예인 줄 알았던 모세가 성소 병사들을 거느린 것을 보고 경악하고, 델릴라는 아론이 옛 동료들을 데려와 속이는 것이라 우긴다. 다말이 화상 입은 발을 보이며 정신을 잃으려 하자 모세는 누가 아내를 이렇게 만들었냐며 살기를 드러내고, 성소 병사들에게 가족을 잡으라 명령한다.</t>
+          <t>모세가 델릴라를 걷어차 쓰러뜨리고 피투성이가 된 다말을 품에 안아 일으킨 뒤 손에 입을 맞춘다. 라반과 네페라는 노예인 줄 알았던 모세가 성소 병사들을 거느린 것을 보고 경악하고, 델릴라는 아론이 옛 동료들을 데려와 속이는 것이라 우긴다. 다말이 정신을 잃으려 하자 모세가 화상 입은 발을 발견하고, 누가 아내를 이렇게 만들었냐며 살기를 드러내고, 성소 병사들에게 가족을 잡으라 명령한다.</t>
         </is>
       </c>
     </row>
@@ -23180,12 +23180,12 @@
         <is>
           <t>★★★
 [키워드] 얼굴불길보복 · 델릴라애원
-[장면] 병사들이 델릴라와 파라오의 얼굴을 불길 앞으로 밀어 넣는다. "Spare me! Anything but my face! Please, I'll do whatever you say!"</t>
+[장면] 병사들이 델릴라와 파라오를 불길 앞으로 끌고 간다. "Spare me! Anything but my face! Please, I'll do whatever you say!" 병사들이 두 사람의 얼굴을 불길 가까이로 밀어 넣는다.</t>
         </is>
       </c>
       <c r="H21" s="243" t="inlineStr">
         <is>
-          <t>모세가 성소 병사들에게 델릴라와 파라오, 라반과 네페라의 얼굴을 신성한 불길 가까이 가져가라 명령하며 다말이 흘린 눈물 한 방울까지 열 배로 갚게 하겠다고 말한다. 병사들이 델릴라와 파라오의 얼굴을 불길 가까이로 밀어 넣자 델릴라는 얼굴만은 안 된다며 애원하고 파라오도 필사적으로 몸부림친다. 바로 그 순간 저택 정문이 열리며 갑옷을 입은 파라오의 병사들이 들어온다.</t>
+          <t>모세가 성소 병사들에게 델릴라와 파라오, 라반과 네페라의 얼굴을 신성한 불길 가까이 가져가라 명령하며 다말이 흘린 눈물 한 방울까지 열 배로 갚게 하겠다고 말한다. 델릴라와 파라오가 불길 앞으로 끌려가 얼굴만은 안 된다며 애원하고 몸부림치자, 병사들이 두 사람의 얼굴을 불길 가까이로 밀어 넣는다. 바로 그 순간 저택 정문이 열리며 갑옷을 입은 파라오의 병사들이 들어온다.</t>
         </is>
       </c>
     </row>
@@ -23232,17 +23232,17 @@
       </c>
       <c r="B23" s="243" t="inlineStr">
         <is>
-          <t>라반 가문의 큰딸. 전생에 파라오의 아내로 살다 대왕비로 책봉되던 날 이복동생의 단검에 죽었고, 3년 전 배필을 정하는 새 의식 아침으로 돌아왔다. 이번에는 가족이 보는 앞에서 비둘기를 노예 구역으로 날려 거지를 남편으로 고른다. 뺨을 맞고, 맨발로 불 위를 걷고, 동생의 발을 씻기고, 목에 칼이 닿는 자리에서도 남편을 부르지 않는다. 그리고 그때마다 왕궁에 재앙이 떨어진다. 이 작품에서 팔리는 그림은 전부 이 인물에게서 나온다.</t>
+          <t>라반 가문의 큰딸. 전생에 파라오의 아내로 살다 대왕비로 책봉되던 날 이복동생의 단검에 죽었고, 3년 전 배필을 정하는 새 의식 아침으로 돌아왔다. 이번에는 가족이 보는 앞에서 비둘기를 노예 구역으로 날려 거지를 남편으로 고른다. 뺨을 맞고, 맨발로 불 위를 걷고, 동생의 발을 씻기고, 목에 칼이 닿는 자리에서도 남편을 부르지 않는다. 그리고 그 뒤에 왕궁에 재앙이 떨어진다. 이 작품에서 팔리는 그림은 전부 이 인물에게서 나온다.</t>
         </is>
       </c>
       <c r="C23" s="243" t="inlineStr">
         <is>
-          <t>Eldest daughter of the house of Laban. In her last life she was Pharaoh's wife and was stabbed by her half-sister the day she was crowned Great Royal Wife, then woke up three years earlier on the morning of the bird ceremony that picks a husband. This time she sends her dove to the slaves' quarter in front of her whole family and marries a beggar. She gets slapped, walks barefoot over fire, washes her sister's feet and takes a blade to her throat without ever calling for him. And every time, a plague hits the palace. Every sellable image in this title comes from her.</t>
+          <t>Eldest daughter of the house of Laban. In her last life she was Pharaoh's wife and was stabbed by her half-sister the day she was crowned Great Royal Wife, then woke up three years earlier on the morning of the bird ceremony that picks a husband. This time she sends her dove to the slaves' quarter in front of her whole family and marries a beggar. She gets slapped, walks barefoot over fire, washes her sister's feet and takes a blade to her throat without ever calling for him. And after each one, a plague hits the palace. Every sellable image in this title comes from her.</t>
         </is>
       </c>
       <c r="D23" s="243" t="inlineStr">
         <is>
-          <t>拉班家的长女。前世身为法老之妻，在被册封为大王妃的当天死于异母妹妹的匕首之下，随后回到三年前择偶鸟祭的清晨。这一世她当着全家人的面把鸽子放向奴隶区，选了一个乞丐做丈夫。她被打耳光、赤脚走火路、给妹妹洗脚、被刀抵住喉咙，也从不呼喊丈夫。而每一次，灾祸都会降临王宫。本作所有能卖的画面，全部来自这个人物。</t>
+          <t>拉班家的长女。前世身为法老之妻，在被册封为大王妃的当天死于异母妹妹的匕首之下，随后回到三年前择偶鸟祭的清晨。这一世她当着全家人的面把鸽子放向奴隶区，选了一个乞丐做丈夫。她被打耳光、赤脚走火路、给妹妹洗脚、被刀抵住喉咙，也从不呼喊丈夫。而在那之后，灾祸便降临王宫。本作所有能卖的画面，全部来自这个人物。</t>
         </is>
       </c>
       <c r="F23" s="247" t="n">
@@ -23267,17 +23267,17 @@
       </c>
       <c r="B24" s="243" t="inlineStr">
         <is>
-          <t>노예 구역에서 돌을 깨는 거지. 실제로는 신의 대언자로, 자기 백성 곁에 있으려고 신분을 숨겼다. 다말이 날린 비둘기가 그의 지팡이에 앉는다. 다말이 다칠 때마다 재앙을 내려 갚고, 아내에게는 대언자라는 사실을 23화에서야 말한다. 혼례 날 붉은 바다를 갈라 다말을 데려가고(EP7), 마지막에 다시 바다를 갈라 백성을 건너게 한 뒤 왕의 군대 위로 바다를 닫는다(EP47~49).</t>
+          <t>노예 구역에서 돌을 깨는 거지. 실제로는 신의 대언자로, 자기 백성 곁에 있으려고 신분을 숨겼다. 다말이 날린 비둘기가 그의 지팡이에 앉는다. 다말이 괴롭힘을 당하면 재앙을 내려 갚고, 아내에게는 대언자라는 사실을 23화에서야 말한다. 혼례 날 붉은 바다를 갈라 다말을 데려가고(EP7), 마지막에 다시 바다를 갈라 백성을 건너게 한 뒤 왕의 군대 위로 바다를 닫는다(EP47~49).</t>
         </is>
       </c>
       <c r="C24" s="243" t="inlineStr">
         <is>
-          <t>A beggar breaking stone in the slaves' quarter. In truth the Prophet of the Lord, hiding his rank to stay beside his people. Tamar's dove lands on his staff. Every time Tamar is hurt he answers with a plague, and he only tells his wife what he is in EP23. On the wedding day he parts the Crimson Sea to take her home (EP7), and in the end he parts it again for his people and closes it over the king's army (EP47-49).</t>
+          <t>A beggar breaking stone in the slaves' quarter. In truth the Prophet of the Lord, hiding his rank to stay beside his people. Tamar's dove lands on his staff. When Tamar is hurt he answers with a plague, and he only tells his wife what he is in EP23. On the wedding day he parts the Crimson Sea to take her home (EP7), and in the end he parts it again for his people and closes it over the king's army (EP47-49).</t>
         </is>
       </c>
       <c r="D24" s="243" t="inlineStr">
         <is>
-          <t>在奴隶区敲石头的乞丐，实为神的代言人，为了留在自己的百姓身边而隐藏身份。塔玛放出的鸽子落在了他的手杖上。塔玛每受一次伤，他就降下灾祸偿还；直到第23集才告诉妻子自己是谁。婚礼当天他分开红海带走塔玛（第7集），最后再次分开大海让百姓渡过，再让海水合拢吞没王军（第47~49集）。</t>
+          <t>在奴隶区敲石头的乞丐，实为神的代言人，为了留在自己的百姓身边而隐藏身份。塔玛放出的鸽子落在了他的手杖上。塔玛受到欺凌，他便降下灾祸偿还；直到第23集才告诉妻子自己是谁。婚礼当天他分开红海带走塔玛（第7集），最后再次分开大海让百姓渡过，再让海水合拢吞没王军（第47~49集）。</t>
         </is>
       </c>
       <c r="F24" s="248" t="n">
@@ -23339,17 +23339,17 @@
       </c>
       <c r="B26" s="243" t="inlineStr">
         <is>
-          <t>신의 피를 이었다고 주장하는 왕국의 통치자. 전생에 다말을 왕비로 두고도 버린 남편이고, 이번 생에서는 델릴라의 매를 받는다. 다말의 얼굴에 낙인을 찍으라고 부추기고(EP16), 노예 해방을 약속하고는 개구리가 사라지자마자 말을 바꾸며, 다말과 라반의 처형을 명한다(EP36). 왕자가 장자 재앙으로 숨을 거두자 아이를 안고 무너져 백성을 보내준다(EP38). 군대를 끌고 바다까지 쫓아왔다가 EP49에서 물벽이 닫히며 군대를 전부 잃고, 홀로 진흙 기슭에 떠밀려 올라와 대왕비 자리를 미끼로 다말을 부르지만 거절당한다.</t>
+          <t>신의 피를 이었다고 주장하는 왕국의 통치자. 전생에 다말의 남편이었고, 이번 생에서는 델릴라의 매를 받는다. 다말의 얼굴에 낙인을 찍으라고 부추기고(EP16), 노예 해방을 약속하고는 개구리가 사라지자마자 말을 바꾸며, 다말과 라반의 처형을 명한다(EP36). 왕자가 장자 재앙으로 숨을 거두자 아이를 안고 무너져 백성을 보내준다(EP38). 군대를 끌고 바다까지 쫓아왔다가 EP49에서 물벽이 닫히며 군대를 전부 잃고, 홀로 진흙 기슭에 떠밀려 올라와 대왕비 자리를 미끼로 다말을 부르지만 거절당한다.</t>
         </is>
       </c>
       <c r="C26" s="243" t="inlineStr">
         <is>
-          <t>Ruler of the kingdom, claiming the blood of the gods. In Tamar's last life he was the husband who made her queen and still threw her away; this time Delilah's hawk lands on him. He eggs on the branding of Tamar's face (EP16), promises to free the slaves and breaks his word the moment the frogs are gone, and orders Tamar and Laban executed (EP36). When the prince dies in the plague of the firstborn he breaks down holding the boy and lets the people go (EP38). He chases them to the sea with his army and loses all of it when the walls of water close in EP49, then washes up alone on the mud and offers Tamar the queen's throne to come back. She refuses.</t>
+          <t>Ruler of the kingdom, claiming the blood of the gods. In Tamar's last life he was her husband; this time Delilah's hawk lands on him. He eggs on the branding of Tamar's face (EP16), promises to free the slaves and breaks his word the moment the frogs are gone, and orders Tamar and Laban executed (EP36). When the prince dies in the plague of the firstborn he breaks down holding the boy and lets the people go (EP38). He chases them to the sea with his army and loses all of it when the walls of water close in EP49, then washes up alone on the mud and offers Tamar the queen's throne to come back. She refuses.</t>
         </is>
       </c>
       <c r="D26" s="243" t="inlineStr">
         <is>
-          <t>自称拥有神之血统的王国统治者。前世他立塔玛为王妃却仍将她抛弃，这一世接住了德莉拉的鹰。他怂恿给塔玛的脸烙印（第16集），答应释放奴隶却在青蛙一消失就翻脸，又下令处死塔玛和拉班（第36集）。王子死于长子之灾后，他抱着孩子崩溃，放百姓离开（第38集）。他率军追到海边，第49集水墙合拢，全军尽失，独自被冲上泥滩，以大王妃之位引诱塔玛回来，被拒绝。</t>
+          <t>自称拥有神之血统的王国统治者。前世他是塔玛的丈夫，这一世接住了德莉拉的鹰。他怂恿给塔玛的脸烙印（第16集），答应释放奴隶却在青蛙一消失就翻脸，又下令处死塔玛和拉班（第36集）。王子死于长子之灾后，他抱着孩子崩溃，放百姓离开（第38集）。他率军追到海边，第49集水墙合拢，全军尽失，独自被冲上泥滩，以大王妃之位引诱塔玛回来，被拒绝。</t>
         </is>
       </c>
       <c r="F26" s="248" t="n">
@@ -23376,17 +23376,17 @@
       </c>
       <c r="B27" s="243" t="inlineStr">
         <is>
-          <t>다말과 델릴라의 아버지. 딸은 가문의 영광을 사 오는 물건이다. 비둘기가 노예 구역으로 날아가자 다말을 쓸모없는 것이라 부르고, 혼인하는 순간 가문과 남남이라고 선언한다(EP5). 다말의 뺨을 때려 쓰러뜨리고(EP13), 델릴라가 언니를 불 위로 걷게 할 때 침묵으로 편든다. 파라오에게 붙잡혀 지하 감옥에 갇히고 광장에서 무릎 꿇려 맞는다(EP30). 처형 직전 모세에게 구해진 뒤(EP36), 해방 행렬 맨 끝에서 가장 무거운 짐을 지고 걸으며 다말에게 네 아비가 아니냐고 매달린다(EP39).</t>
+          <t>다말과 델릴라의 아버지. 딸은 가문의 영광을 사 오는 물건이다. 비둘기가 노예 구역으로 날아가자(EP2) 다말을 쓸모없는 것이라 부르고(EP4), 혼인하는 순간 가문과 남남이라고 선언한다(EP5). 다말의 뺨을 때려 쓰러뜨리고(EP13), 델릴라가 언니를 불 위로 걷게 할 때 침묵으로 편든다. 파라오에게 붙잡혀 지하 감옥에 갇히고 광장에서 무릎 꿇려 맞는다(EP30). 처형 직전 모세에게 구해진 뒤(EP36), 해방 행렬 맨 끝에서 가장 무거운 짐을 지고 걸으며 다말에게 네 아비가 아니냐고 매달린다(EP39).</t>
         </is>
       </c>
       <c r="C27" s="243" t="inlineStr">
         <is>
-          <t>Father of Tamar and Delilah. A daughter, to him, is a thing that buys glory for the house. When the dove flies to the slaves' quarter he calls Tamar useless and declares her nothing to the family the moment she marries (EP5). He slaps her to the ground (EP13) and sides with Delilah in silence while she makes her sister walk on fire. Pharaoh throws him in the dungeon and has him beaten on his knees in the square (EP30). Saved by Moses seconds before execution (EP36), he ends up at the tail of the freed people's column carrying the heaviest load, begging Tamar to remember he is still her father (EP39).</t>
+          <t>Father of Tamar and Delilah. A daughter, to him, is a thing that buys glory for the house. When the dove flies to the slaves' quarter (EP2) he calls Tamar useless (EP4) and declares her nothing to the family the moment she marries (EP5). He slaps her to the ground (EP13) and sides with Delilah in silence while she makes her sister walk on fire. Pharaoh throws him in the dungeon and has him beaten on his knees in the square (EP30). Saved by Moses seconds before execution (EP36), he ends up at the tail of the freed people's column carrying the heaviest load, begging Tamar to remember he is still her father (EP39).</t>
         </is>
       </c>
       <c r="D27" s="243" t="inlineStr">
         <is>
-          <t>塔玛和德莉拉的父亲。在他眼里女儿是为家族换取荣耀的物件。鸽子飞向奴隶区后他骂塔玛没用，宣布她一旦成婚就与家族再无关系（第5集）。他一巴掌把塔玛打倒在地（第13集），德莉拉逼姐姐走火路时他以沉默站在小女儿一边。后被法老关进地牢，在广场上跪着挨打（第30集）。处刑前一刻被摩西所救（第36集），最后在解放队伍的末尾背着最重的行李，哀求塔玛别忘了他还是她的父亲（第39集）。</t>
+          <t>塔玛和德莉拉的父亲。在他眼里女儿是为家族换取荣耀的物件。鸽子飞向奴隶区后（第2集）他骂塔玛没用（第4集），宣布她一旦成婚就与家族再无关系（第5集）。他一巴掌把塔玛打倒在地（第13集），德莉拉逼姐姐走火路时他以沉默站在小女儿一边。后被法老关进地牢，在广场上跪着挨打（第30集）。处刑前一刻被摩西所救（第36集），最后在解放队伍的末尾背着最重的行李，哀求塔玛别忘了他还是她的父亲（第39集）。</t>
         </is>
       </c>
       <c r="F27" s="248" t="n">
@@ -23495,7 +23495,7 @@
       </c>
       <c r="H31" s="243" t="inlineStr">
         <is>
-          <t>델릴라가 지하 감옥에 갇힌 다말을 찾아와 조롱하며 발을 씻기라 명령하고, 다말은 아버지를 살리기 위해 무릎 꿇고 델릴라의 발을 씻긴다. 하녀들은 그 모습을 보며 비웃고, 델릴라는 오랫동안 꿈꿔온 순간이라며 만족스러워한다. 새벽이 되자 왕궁 전체에 흙먼지가 이로 변해 퍼지고, 델릴라의 몸에 이가 들러붙어 비명을 지른다.</t>
+          <t>델릴라가 지하 감옥에 갇힌 다말을 찾아와 조롱하고, 하녀들이 다말을 무릎 꿇리자 다말은 아버지를 살리기 위해 델릴라의 발을 씻긴다. 하녀들은 그 모습을 보며 비웃고, 델릴라는 오랫동안 꿈꿔온 순간이라며 만족스러워한다. 새벽이 되자 왕궁 전체에 흙먼지가 이로 변해 퍼지고, 델릴라의 몸에 이가 들러붙어 비명을 지른다.</t>
         </is>
       </c>
     </row>
@@ -23518,7 +23518,7 @@
       </c>
       <c r="H32" s="243" t="inlineStr">
         <is>
-          <t>이 재앙에 왕국 최고의 술사들도 손을 놓고, 파라오는 분노한다. 지하 감옥에서 낯선 얼굴로 변신한 모세가 다말에게 손을 내밀며 성소로 돌아가자고 청하지만, 다말은 아버지를 두고 갈 수 없다며 거절한다. 모세는 말없이 돌아서 사라졌다가, 아무도 없는 곳에서 원래 얼굴로 돌아와 다말을 자신의 방식대로 지키겠다고 다짐한다.</t>
+          <t>이 재앙에 왕국 최고의 술사들도 손을 놓고, 파라오는 분노한다. 지하 감옥에서 낯선 얼굴로 변신한 모세가 다말에게 손을 내밀며 성소로 돌아가자고 청하지만, 다말은 아버지를 두고 갈 수 없다며 거절한다. 모세는 그대의 뜻을 존중하겠다며 돌아서 사라졌다가, 아무도 없는 곳에서 원래 얼굴로 돌아와 다말을 자신의 방식대로 지키겠다고 다짐한다.</t>
         </is>
       </c>
     </row>
@@ -23547,7 +23547,7 @@
       </c>
       <c r="H33" s="243" t="inlineStr">
         <is>
-          <t>왕궁 병사들이 광장에서 라반을 무릎 꿇리고 때리자 다말이 몸부림치며 막아서지만, 파라오는 침묵하면 아비를 버리는 것이라 다그친다. 다말이 굴복하지 않겠다 외치자 하늘에서 거대한 우박이 쏟아지고, 라반을 때린 근위대장과 다말을 조롱한 델릴라만 정확히 맞아 쓰러진다. 군중이 신이 다말의 편이라 웅성거리자 파라오는 다말을 다시 지하 감옥에 가두라 명하고, 네페라가 다말에게 복수를 다짐한다.</t>
+          <t>광장에서 근위대장이 쇠사슬에 묶인 라반을 무릎 꿇리고 때리자 다말이 몸부림치며 막아서지만, 파라오는 침묵하면 아비를 버리는 것이라 다그친다. 다말이 굴복하지 않겠다 외치자 하늘에서 거대한 우박이 쏟아지고, 라반을 때린 근위대장과 다말을 조롱한 델릴라만 정확히 맞아 쓰러진다. 군중이 신이 다말의 편이라 웅성거리자 파라오는 다말을 다시 지하 감옥에 가두라 명하고, 네페라가 다말에게 복수를 다짐한다.</t>
         </is>
       </c>
     </row>
@@ -23712,17 +23712,17 @@
       </c>
       <c r="B40" s="243" t="inlineStr">
         <is>
-          <t>펜던트를 되찾으려 피투성이 손으로 바닥을 기는 다말의 턱을 델릴라가 잡고, 시뻘겋게 달군 태양 낙인을 얼굴에 가져다 댄다. 파라오가 소리친다. "Burn her! Make that traitor suffer!" 낙인이 내려오는 순간 모래폭풍이 낙인을 쳐내 돌기둥에 박는다. "Get away from her!"</t>
+          <t>피투성이 손으로 바닥을 기어 펜던트를 되찾은 다말의 턱을 델릴라가 잡고, 시뻘겋게 달군 태양 낙인을 얼굴에 가져다 댄다. 파라오가 소리친다. "Burn her! Make that traitor suffer!" 낙인이 내려오는 순간 모래폭풍이 낙인을 쳐내 돌기둥에 박는다. "Get away from her!"</t>
         </is>
       </c>
       <c r="C40" s="243" t="inlineStr">
         <is>
-          <t>Tamar crawls across the floor with bloodied hands to get her pendant back. Delilah grabs her jaw and brings a red-hot sun-shaped brand to her face while Pharaoh shouts, "Burn her! Make that traitor suffer!" As the brand comes down, a sandstorm knocks it out of Delilah's hand and buries it in a stone pillar. "Get away from her!"</t>
+          <t>Tamar crawls across the floor with bloodied hands and gets her pendant back. Delilah grabs her jaw and brings a red-hot sun-shaped brand to her face while Pharaoh shouts, "Burn her! Make that traitor suffer!" As the brand comes down, a sandstorm knocks it out of Delilah's hand and buries it in a stone pillar. "Get away from her!"</t>
         </is>
       </c>
       <c r="D40" s="243" t="inlineStr">
         <is>
-          <t>塔玛用血淋淋的双手在地上爬着去捡回吊坠，德莉拉掐住她的下巴，把烧红的太阳烙铁按向她的脸，法老在旁大喊“烧她！让那个叛徒受苦！”烙铁落下的瞬间，沙暴把烙铁打飞，深深钉进石柱。“离她远点！”</t>
+          <t>塔玛用血淋淋的双手爬过地面捡回吊坠，德莉拉掐住她的下巴，把烧红的太阳烙铁按向她的脸，法老在旁大喊“烧她！让那个叛徒受苦！”烙铁落下的瞬间，沙暴把烙铁打飞，深深钉进石柱。“离她远点！”</t>
         </is>
       </c>
       <c r="F40" s="247" t="n">
@@ -23747,17 +23747,17 @@
       </c>
       <c r="B41" s="243" t="inlineStr">
         <is>
-          <t>모세가 명령한다. "Hold their faces close to the sacred fire." 병사들이 델릴라와 파라오의 얼굴을 다말이 걸었던 불길 앞으로 밀어 넣는다. 델릴라가 비명을 지른다. "Spare me! Anything but my face! Please, I'll do whatever you say!"</t>
+          <t>모세가 명령한다. "Hold their faces close to the sacred fire." 병사들이 델릴라와 파라오를 다말이 걸었던 불길 앞으로 끌고 간다. 델릴라가 비명을 지른다. "Spare me! Anything but my face! Please, I'll do whatever you say!" 병사들이 두 사람의 얼굴을 불길 가까이로 밀어 넣는다.</t>
         </is>
       </c>
       <c r="C41" s="243" t="inlineStr">
         <is>
-          <t>Moses gives the order: "Hold their faces close to the sacred fire." The soldiers shove Delilah's and Pharaoh's faces toward the same flames Tamar walked through. Delilah screams, "Spare me! Anything but my face! Please, I'll do whatever you say!"</t>
+          <t>Moses gives the order: "Hold their faces close to the sacred fire." The soldiers drag Delilah and Pharaoh to the same flames Tamar walked through. Delilah screams, "Spare me! Anything but my face! Please, I'll do whatever you say!" Then the soldiers shove both faces toward the fire.</t>
         </is>
       </c>
       <c r="D41" s="243" t="inlineStr">
         <is>
-          <t>摩西下令：“把他们的脸按到圣火前。”士兵把德莉拉和法老的脸推向塔玛走过的那条火路。德莉拉尖叫：“饶了我！别毁我的脸！求你，你说什么我都照做！”</t>
+          <t>摩西下令：“把他们的脸按到圣火前。”士兵把德莉拉和法老拖到塔玛走过的那条火路前。德莉拉尖叫：“饶了我！别毁我的脸！求你，你说什么我都照做！”随后士兵把两人的脸推向火焰。</t>
         </is>
       </c>
       <c r="F41" s="247" t="n">
@@ -23837,7 +23837,7 @@
         <is>
           <t>★★
 [키워드] 미리암정체 · 손치유 · 키스
-[장면] 모세가 다말의 손바닥 상처를 어루만지자 상처가 낫는다. 다말이 달려가 안기고 두 사람이 입을 맞춘다.</t>
+[장면] 다말이 달려가 안기고, 모세가 다말의 손바닥 상처를 어루만지자 상처가 낫는다. 두 사람이 입을 맞춘다.</t>
         </is>
       </c>
       <c r="H43" s="243" t="inlineStr">
@@ -23889,17 +23889,17 @@
       </c>
       <c r="B45" s="243" t="inlineStr">
         <is>
-          <t>물벽이 무너져 왕의 군대를 삼킨다. 델릴라가 부서진 전차 잔해를 타고 진흙투성이로 다말의 발치까지 기어온다. 다말이 델릴라의 손목에서 대왕비의 팔찌를 빼내 웅덩이에 던진다. "Give it back! That's the Great Royal Wife's bracelet!" 다말이 귓가에 말한다. "Live, and pay the price."</t>
+          <t>물벽이 무너져 왕의 군대를 삼킨다. 델릴라가 부서진 전차 잔해를 타고 진흙투성이로 다말의 발치까지 기어온다. 다말이 델릴라의 손목에서 대왕비의 팔찌를 빼낸다. "Give it back! That's the Great Royal Wife's bracelet!" 다말이 팔찌를 웅덩이에 던지고 귓가에 말한다. "Live, and pay the price."</t>
         </is>
       </c>
       <c r="C45" s="243" t="inlineStr">
         <is>
-          <t>The walls of water collapse and swallow the king's army. Delilah crawls over the wreckage of a chariot, caked in mud, to Tamar's feet. Tamar rips the Great Royal Wife's bracelet off her wrist and throws it into a puddle. "Give it back! That's the Great Royal Wife's bracelet!" Tamar bends to her ear: "Live, and pay the price."</t>
+          <t>The walls of water collapse and swallow the king's army. Delilah crawls over the wreckage of a chariot, caked in mud, to Tamar's feet. Tamar rips the Great Royal Wife's bracelet off her wrist. "Give it back! That's the Great Royal Wife's bracelet!" Tamar throws it into a puddle and bends to her ear: "Live, and pay the price."</t>
         </is>
       </c>
       <c r="D45" s="243" t="inlineStr">
         <is>
-          <t>水墙崩塌，吞没王军。德莉拉爬过破碎的战车残骸，满身泥浆地爬到塔玛脚边。塔玛从她手腕上扯下大王妃手镯扔进水洼。“还给我！那是大王妃的手镯！”塔玛俯身在她耳边说：“活着，付出代价。”</t>
+          <t>水墙崩塌，吞没王军。德莉拉爬过破碎的战车残骸，满身泥浆地爬到塔玛脚边。塔玛从她手腕上扯下大王妃手镯。“还给我！那是大王妃的手镯！”塔玛把手镯扔进水洼，俯身在她耳边说：“活着，付出代价。”</t>
         </is>
       </c>
       <c r="F45" s="247" t="n">
@@ -23951,7 +23951,7 @@
       </c>
       <c r="H47" s="243" t="inlineStr">
         <is>
-          <t>붉은 바다 앞에 갇힌 백성들은 모세의 멱살을 잡고 원망을 쏟아내고, 다말이 나서서 사람들을 진정시킨다. 뒤쫓아온 왕실군이 행렬 후미까지 따라붙고, 전차 위의 델릴라가 군중 사이에서 다말을 발견한다. 델릴라는 차갑게 웃으며 다말을 찾아냈다고 말한다.</t>
+          <t>붉은 바다 앞에 갇힌 백성 하나가 모세의 멱살을 잡고 원망을 쏟아내자, 다말이 나서서 사람들을 진정시킨다. 뒤쫓아온 왕실군이 행렬 후미까지 따라붙고, 전차 위의 델릴라가 군중 사이에서 다말을 발견한다. 델릴라는 차갑게 웃으며 다말을 찾아냈다고 말한다.</t>
         </is>
       </c>
     </row>

</xml_diff>